<commit_message>
Added asl to the namespace registry
</commit_message>
<xml_diff>
--- a/docs/namespace-registry/pds-namespace-registry.xlsx
+++ b/docs/namespace-registry/pds-namespace-registry.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AA7Ontologies\A01PDS4\03_Namespaces\NameSpaceRegistry\260218_ops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AA7Ontologies\A01PDS4\03_Namespaces\NameSpaceRegistry\260218b_asl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843F5DB0-16FE-4F32-A921-62CF244B861B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6D14FF-ABF3-4A63-9BE4-53E4B71DA04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{FAC3036B-2C0F-0A46-BDED-22E3426EC150}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="495">
   <si>
     <t>Namespace Id (1)</t>
   </si>
@@ -247,9 +247,6 @@
   </si>
   <si>
     <t>The Particle dictionary contains classes that describe the composition of multidimensional particle data consisting of Array (and Array subclass) data objects.</t>
-  </si>
-  <si>
-    <t>Namespace for the Operations dictionary.</t>
   </si>
   <si>
     <t>Namespace for the PPI node's dictionary.</t>
@@ -1496,7 +1493,25 @@
     <t>Sophia Conover</t>
   </si>
   <si>
-    <t>sophia.n.conover@jpl.nasa.gov</t>
+    <t>asl</t>
+  </si>
+  <si>
+    <t>Mars Missions Analogue Sample Library</t>
+  </si>
+  <si>
+    <t>Mars Missions Analogue Sample Library metadata</t>
+  </si>
+  <si>
+    <t>Thomas Cornet</t>
+  </si>
+  <si>
+    <t>thomas.cornet at esa.int</t>
+  </si>
+  <si>
+    <t>sophia.n.conover at jpl.nasa.gov</t>
+  </si>
+  <si>
+    <t>Operations metadata appended to PDS4 metadata in order to support PDS Core Services, such as the Registry.</t>
   </si>
 </sst>
 </file>
@@ -1637,10 +1652,6 @@
     <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1651,9 +1662,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1668,6 +1676,13 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1986,7 +2001,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr defaultColWidth="11.20703125" defaultRowHeight="16" x14ac:dyDescent="0.8"/>
   <cols>
     <col min="1" max="1" width="14.2890625" style="4" customWidth="1"/>
@@ -1995,12 +2010,12 @@
     <col min="4" max="4" width="12.2890625" style="4" customWidth="1"/>
     <col min="5" max="5" width="23" style="4" customWidth="1"/>
     <col min="6" max="6" width="31.6640625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="16.20703125" style="15" customWidth="1"/>
+    <col min="7" max="7" width="16.20703125" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A1" s="12" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B1" s="12">
         <v>46071</v>
@@ -2011,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -2020,12 +2035,12 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="14" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2038,7 +2053,7 @@
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="17"/>
+      <c r="G3" s="15"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A4" s="7" t="s">
@@ -2059,7 +2074,7 @@
       <c r="F4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="16">
         <v>41002</v>
       </c>
     </row>
@@ -2072,7 +2087,7 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="17"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A6" s="7" t="s">
@@ -2093,7 +2108,7 @@
       <c r="F6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="16">
         <v>42811</v>
       </c>
     </row>
@@ -2116,30 +2131,30 @@
       <c r="F7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="16">
         <v>42922</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A8" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>255</v>
-      </c>
-      <c r="G8" s="18">
+      <c r="G8" s="16">
         <v>44426</v>
       </c>
     </row>
@@ -2162,7 +2177,7 @@
       <c r="F9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="16">
         <v>42277</v>
       </c>
     </row>
@@ -2185,7 +2200,7 @@
       <c r="F10" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="16">
         <v>42811</v>
       </c>
     </row>
@@ -2194,7 +2209,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>37</v>
@@ -2208,7 +2223,7 @@
       <c r="F11" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="16">
         <v>44132</v>
       </c>
     </row>
@@ -2221,14 +2236,14 @@
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="17"/>
+      <c r="G12" s="15"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A13" s="7" t="s">
         <v>38</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>42</v>
@@ -2242,19 +2257,19 @@
       <c r="F13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="16">
         <v>42118</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A14" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>416</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>417</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>13</v>
@@ -2265,7 +2280,7 @@
       <c r="F14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="16">
         <v>45680</v>
       </c>
     </row>
@@ -2274,7 +2289,7 @@
         <v>43</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>46</v>
@@ -2288,7 +2303,7 @@
       <c r="F15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="16">
         <v>41002</v>
       </c>
     </row>
@@ -2311,19 +2326,19 @@
       <c r="F16" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="18">
+      <c r="G16" s="16">
         <v>42299</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A17" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>235</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>13</v>
@@ -2334,7 +2349,7 @@
       <c r="F17" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G17" s="18">
+      <c r="G17" s="16">
         <v>44329</v>
       </c>
     </row>
@@ -2357,30 +2372,30 @@
       <c r="F18" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="16">
         <v>41435</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="64" x14ac:dyDescent="0.8">
       <c r="A19" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E19" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>248</v>
-      </c>
-      <c r="G19" s="18">
+      <c r="G19" s="16">
         <v>44398</v>
       </c>
     </row>
@@ -2403,7 +2418,7 @@
       <c r="F20" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="16">
         <v>42124</v>
       </c>
     </row>
@@ -2426,7 +2441,7 @@
       <c r="F21" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="18">
+      <c r="G21" s="16">
         <v>41002</v>
       </c>
     </row>
@@ -2435,7 +2450,7 @@
         <v>64</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>65</v>
@@ -2449,42 +2464,42 @@
       <c r="F22" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G22" s="18">
+      <c r="G22" s="16">
         <v>43734</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A23" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E23" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="G23" s="18">
+      <c r="G23" s="16">
         <v>44333</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A24" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>13</v>
@@ -2495,7 +2510,7 @@
       <c r="F24" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G24" s="18">
+      <c r="G24" s="16">
         <v>42650</v>
       </c>
     </row>
@@ -2504,7 +2519,7 @@
         <v>66</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>67</v>
@@ -2518,19 +2533,19 @@
       <c r="F25" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G25" s="18">
+      <c r="G25" s="16">
         <v>43734</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="80" x14ac:dyDescent="0.8">
       <c r="A26" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>13</v>
@@ -2541,7 +2556,7 @@
       <c r="F26" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G26" s="18">
+      <c r="G26" s="16">
         <v>44257</v>
       </c>
     </row>
@@ -2550,7 +2565,7 @@
         <v>68</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>71</v>
@@ -2564,54 +2579,54 @@
       <c r="F27" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="G27" s="18">
+      <c r="G27" s="16">
         <v>44110</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+    <row r="28" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A28" s="7" t="s">
-        <v>72</v>
+        <v>486</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>225</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>73</v>
+        <v>494</v>
       </c>
       <c r="D28" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E28" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>493</v>
+      </c>
+      <c r="G28" s="16">
+        <v>41002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A29" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G28" s="18">
+      <c r="G29" s="16">
         <v>42118</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="14" customFormat="1" x14ac:dyDescent="0.8">
-      <c r="A29" s="13" t="s">
-        <v>487</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>488</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>489</v>
-      </c>
-      <c r="G29" s="19">
-        <v>41002</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.8">
@@ -2620,7 +2635,7 @@
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>13</v>
@@ -2631,19 +2646,19 @@
       <c r="F30" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G30" s="18">
+      <c r="G30" s="16">
         <v>41002</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A31" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>13</v>
@@ -2654,19 +2669,19 @@
       <c r="F31" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G31" s="18">
+      <c r="G31" s="16">
         <v>43734</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A32" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="C32" s="7" t="s">
         <v>482</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>483</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>13</v>
@@ -2677,111 +2692,111 @@
       <c r="F32" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G32" s="18">
+      <c r="G32" s="16">
         <v>45924</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A33" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E33" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F33" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="G33" s="18">
+      <c r="G33" s="16">
         <v>41002</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A34" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>318</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>319</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E34" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G34" s="18">
+      <c r="G34" s="16">
         <v>44943</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A35" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E35" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F35" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F35" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G35" s="18">
+      <c r="G35" s="16">
         <v>41589</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A36" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>89</v>
-      </c>
       <c r="C36" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E36" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G36" s="18">
+      <c r="G36" s="16">
         <v>42870</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A37" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B37" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="C37" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>95</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>13</v>
@@ -2792,102 +2807,102 @@
       <c r="F37" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="G37" s="18">
+      <c r="G37" s="16">
         <v>44110</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A38" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
-      <c r="G38" s="17"/>
+      <c r="G38" s="15"/>
     </row>
     <row r="39" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A39" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E39" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="F39" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="G39" s="16">
+        <v>44791</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="23" customFormat="1" ht="32" x14ac:dyDescent="0.8">
+      <c r="A40" s="21" t="s">
+        <v>488</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>489</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>490</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E40" s="21" t="s">
+        <v>491</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>492</v>
+      </c>
+      <c r="G40" s="22">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A41" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>313</v>
       </c>
-      <c r="C39" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G39" s="18">
-        <v>44791</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A40" s="7" t="s">
+      <c r="C41" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E40" s="7" t="s">
+      <c r="D41" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F41" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F40" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G40" s="18">
+      <c r="G41" s="16">
         <v>42089</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="96" x14ac:dyDescent="0.8">
-      <c r="A41" s="7" t="s">
+    <row r="42" spans="1:7" ht="96" x14ac:dyDescent="0.8">
+      <c r="A42" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B42" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="C42" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G41" s="18">
-        <v>44329</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A42" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>244</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>245</v>
-      </c>
       <c r="D42" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>50</v>
@@ -2895,275 +2910,275 @@
       <c r="F42" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G42" s="18">
-        <v>44385</v>
+      <c r="G42" s="16">
+        <v>44329</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A43" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G43" s="16">
+        <v>44385</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A44" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>322</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="7" t="s">
+      <c r="D44" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="F44" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="F43" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G43" s="18">
+      <c r="G44" s="16">
         <v>45013</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A44" s="7" t="s">
+    <row r="45" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A45" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E44" s="7" t="s">
+      <c r="D45" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="F45" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="F44" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G44" s="18">
+      <c r="G45" s="16">
         <v>44426</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A45" s="7" t="s">
-        <v>471</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>472</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>473</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>474</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>475</v>
-      </c>
-      <c r="G45" s="18">
-        <v>45868</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="48" x14ac:dyDescent="0.8">
       <c r="A46" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>473</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="G46" s="16">
+        <v>45868</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A47" s="7" t="s">
+        <v>475</v>
+      </c>
+      <c r="B47" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="C47" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D47" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="F47" s="8" t="s">
         <v>478</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>480</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>479</v>
-      </c>
-      <c r="G46" s="18">
+      <c r="G47" s="16">
         <v>45923</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A47" s="7" t="s">
-        <v>430</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="C47" s="7" t="s">
-        <v>439</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E47" s="7" t="s">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A48" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F48" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F47" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G47" s="18">
+      <c r="G48" s="16">
         <v>45742</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A48" s="7" t="s">
+    <row r="49" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A49" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B49" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="C49" s="7" t="s">
         <v>279</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>280</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E48" s="7" t="s">
+      <c r="D49" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="F49" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="F48" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="G48" s="18">
+      <c r="G49" s="16">
         <v>44707</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A49" s="7" t="s">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A50" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B49" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E49" s="7" t="s">
+      <c r="D50" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E50" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F49" s="7" t="s">
+      <c r="F50" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G49" s="18">
+      <c r="G50" s="16">
         <v>44193</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A50" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E50" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="G50" s="18">
-        <v>44735</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A51" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="G51" s="16">
+        <v>44735</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A52" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="C52" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="D52" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E52" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="C51" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E51" s="7" t="s">
+      <c r="F52" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="F51" s="7" t="s">
-        <v>268</v>
-      </c>
-      <c r="G51" s="18">
+      <c r="G52" s="16">
         <v>44426</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A52" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="B52" s="7" t="s">
-        <v>292</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G52" s="18">
-        <v>42119</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A53" s="7" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>110</v>
+        <v>291</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="G53" s="18">
-        <v>41837</v>
+        <v>90</v>
+      </c>
+      <c r="G53" s="16">
+        <v>42119</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A54" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B54" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="C54" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C54" s="7" t="s">
-        <v>112</v>
-      </c>
       <c r="D54" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E54" s="7" t="s">
         <v>44</v>
@@ -3171,275 +3186,275 @@
       <c r="F54" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G54" s="18">
+      <c r="G54" s="16">
         <v>41837</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A55" s="7" t="s">
-        <v>411</v>
+        <v>108</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>412</v>
+        <v>109</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>413</v>
+        <v>111</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>310</v>
+        <v>44</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G55" s="18">
-        <v>45612</v>
+        <v>45</v>
+      </c>
+      <c r="G55" s="16">
+        <v>41837</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A56" s="7" t="s">
-        <v>260</v>
+        <v>410</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>262</v>
+        <v>411</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>263</v>
+        <v>412</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>90</v>
+        <v>309</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G56" s="18">
-        <v>44608</v>
+        <v>310</v>
+      </c>
+      <c r="G56" s="16">
+        <v>45612</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A57" s="7" t="s">
-        <v>324</v>
+        <v>259</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>325</v>
+        <v>261</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>326</v>
+        <v>262</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>327</v>
+        <v>89</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="G57" s="18">
-        <v>44957</v>
+        <v>90</v>
+      </c>
+      <c r="G57" s="16">
+        <v>44608</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A58" s="7" t="s">
-        <v>242</v>
+        <v>323</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>261</v>
+        <v>324</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>243</v>
+        <v>325</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>90</v>
+        <v>326</v>
       </c>
       <c r="F58" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G58" s="18">
-        <v>44333</v>
+        <v>327</v>
+      </c>
+      <c r="G58" s="16">
+        <v>44957</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A59" s="7" t="s">
-        <v>113</v>
+        <v>241</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>294</v>
+        <v>260</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>114</v>
+        <v>242</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E59" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F59" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="F59" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G59" s="18">
-        <v>43935</v>
+      <c r="G59" s="16">
+        <v>44333</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A60" s="7" t="s">
-        <v>335</v>
+        <v>112</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>336</v>
+        <v>293</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>337</v>
+        <v>113</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>310</v>
+        <v>89</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G60" s="18">
-        <v>45146</v>
+        <v>90</v>
+      </c>
+      <c r="G60" s="16">
+        <v>43935</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A61" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="G61" s="16">
+        <v>45146</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A62" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="C62" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B61" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E61" s="7" t="s">
+      <c r="D62" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E62" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F61" s="7" t="s">
+      <c r="F62" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G61" s="18">
+      <c r="G62" s="16">
         <v>41600</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A62" s="7" t="s">
-        <v>431</v>
-      </c>
-      <c r="B62" s="7" t="s">
-        <v>435</v>
-      </c>
-      <c r="C62" s="7" t="s">
-        <v>438</v>
-      </c>
-      <c r="D62" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E62" s="7" t="s">
+    <row r="63" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A63" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F63" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F62" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G62" s="18">
+      <c r="G63" s="16">
         <v>45742</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A63" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="C63" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D63" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E63" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="F63" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="G63" s="18">
-        <v>42220</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A64" s="7" t="s">
-        <v>329</v>
+        <v>116</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>330</v>
+        <v>295</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>331</v>
+        <v>117</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>310</v>
+        <v>50</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G64" s="18">
-        <v>44951</v>
+        <v>51</v>
+      </c>
+      <c r="G64" s="16">
+        <v>42220</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A65" s="7" t="s">
-        <v>119</v>
+        <v>328</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>293</v>
+        <v>329</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>120</v>
+        <v>330</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>40</v>
+        <v>309</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G65" s="18">
-        <v>42158</v>
+        <v>310</v>
+      </c>
+      <c r="G65" s="16">
+        <v>44951</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A66" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="C66" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B66" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="C66" s="7" t="s">
-        <v>121</v>
-      </c>
       <c r="D66" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E66" s="7" t="s">
         <v>40</v>
@@ -3447,218 +3462,218 @@
       <c r="F66" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G66" s="18">
+      <c r="G66" s="16">
         <v>42158</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A67" s="7" t="s">
-        <v>315</v>
+        <v>118</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>316</v>
+        <v>292</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>317</v>
+        <v>120</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>310</v>
+        <v>40</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G67" s="18">
-        <v>44833</v>
+        <v>41</v>
+      </c>
+      <c r="G67" s="16">
+        <v>42158</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A68" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="F68" s="7" t="s">
+        <v>310</v>
+      </c>
+      <c r="G68" s="16">
+        <v>44833</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A69" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="B69" s="7" t="s">
         <v>286</v>
       </c>
-      <c r="B68" s="7" t="s">
+      <c r="C69" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="C68" s="7" t="s">
-        <v>288</v>
-      </c>
-      <c r="D68" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E68" s="7" t="s">
+      <c r="D69" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="F69" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="F68" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="G68" s="18">
+      <c r="G69" s="16">
         <v>44713</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A69" s="7" t="s">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A70" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C70" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="B69" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="C69" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E69" s="7" t="s">
+      <c r="D70" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F70" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F69" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="G69" s="18">
+      <c r="G70" s="16">
         <v>43871</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A70" s="7" t="s">
+    <row r="71" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A71" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E71" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D70" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E70" s="7" t="s">
+      <c r="F71" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="F70" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="G70" s="18">
+      <c r="G71" s="16">
         <v>44643</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A71" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="B71" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>283</v>
-      </c>
-      <c r="D71" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E71" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="F71" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="G71" s="18">
-        <v>44713</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A72" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="F72" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="G72" s="16">
+        <v>44713</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A73" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E73" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B72" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="D72" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E72" s="7" t="s">
+      <c r="F73" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F72" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="G72" s="18">
+      <c r="G73" s="16">
         <v>41771</v>
       </c>
     </row>
-    <row r="73" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A73" s="7" t="s">
+    <row r="74" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A74" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="C74" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="B73" s="7" t="s">
-        <v>484</v>
-      </c>
-      <c r="C73" s="7" t="s">
-        <v>486</v>
-      </c>
-      <c r="D73" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E73" s="7" t="s">
+      <c r="D74" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="F74" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="F73" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="G73" s="18">
+      <c r="G74" s="16">
         <v>45966</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A74" s="7" t="s">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A75" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B75" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="B74" s="7" t="s">
+      <c r="C75" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="C74" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="D74" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E74" s="7" t="s">
+      <c r="D75" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="F75" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="F74" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="G74" s="18">
+      <c r="G75" s="16">
         <v>45014</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A75" s="7" t="s">
-        <v>429</v>
-      </c>
-      <c r="B75" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="C75" s="7" t="s">
-        <v>437</v>
-      </c>
-      <c r="D75" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E75" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="F75" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G75" s="18">
-        <v>45742</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.8">
+    <row r="76" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A76" s="7" t="s">
         <v>428</v>
       </c>
@@ -3669,76 +3684,76 @@
         <v>436</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E76" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F76" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F76" s="8" t="s">
+      <c r="G76" s="16">
+        <v>45742</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A77" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="G77" s="16">
+        <v>45742</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A78" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="G76" s="18">
-        <v>45742</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A77" s="7" t="s">
+      <c r="C78" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="B77" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C77" s="7" t="s">
+      <c r="D78" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E78" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="D77" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E77" s="7" t="s">
+      <c r="F78" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F77" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G77" s="18">
+      <c r="G78" s="16">
         <v>45914</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A78" s="7" t="s">
-        <v>343</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="C78" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="D78" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E78" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F78" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G78" s="18">
-        <v>45203</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A79" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B79" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="B79" s="7" t="s">
-        <v>346</v>
-      </c>
       <c r="C79" s="7" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>40</v>
@@ -3746,1656 +3761,1679 @@
       <c r="F79" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G79" s="18">
+      <c r="G79" s="16">
         <v>45203</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A80" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G80" s="16">
+        <v>45203</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A81" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="B81" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="C81" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E81" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="D80" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E80" s="7" t="s">
+      <c r="F81" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="F80" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="G80" s="18">
+      <c r="G81" s="16">
         <v>44700</v>
       </c>
     </row>
-    <row r="81" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A81" s="7" t="s">
+    <row r="82" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A82" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="B82" s="7" t="s">
         <v>355</v>
       </c>
-      <c r="B81" s="7" t="s">
+      <c r="C82" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="C81" s="7" t="s">
+      <c r="D82" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="F82" s="9" t="s">
         <v>357</v>
       </c>
-      <c r="D81" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E81" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="G81" s="18">
+      <c r="G82" s="16">
         <v>45489</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A82" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="B82" s="7" t="s">
-        <v>351</v>
-      </c>
-      <c r="C82" s="7" t="s">
-        <v>354</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>353</v>
-      </c>
-      <c r="F82" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="G82" s="18">
-        <v>45031</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A83" s="7" t="s">
-        <v>126</v>
+        <v>349</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>301</v>
+        <v>350</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>129</v>
+        <v>353</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>127</v>
+        <v>352</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="G83" s="18">
-        <v>43788</v>
+        <v>351</v>
+      </c>
+      <c r="G83" s="16">
+        <v>45031</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A84" s="7" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B84" s="7" t="s">
-        <v>452</v>
+        <v>300</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D84" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E84" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F84" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="F84" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G84" s="18">
+      <c r="G84" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A85" s="7" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E85" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G85" s="18">
+        <v>130</v>
+      </c>
+      <c r="G85" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A86" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B86" s="7" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D86" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E86" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F86" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G86" s="18">
+        <v>130</v>
+      </c>
+      <c r="G86" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A87" s="7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E87" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G87" s="18">
+        <v>130</v>
+      </c>
+      <c r="G87" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A88" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B88" s="7" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D88" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E88" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F88" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G88" s="18">
+        <v>130</v>
+      </c>
+      <c r="G88" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A89" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G89" s="18">
+        <v>130</v>
+      </c>
+      <c r="G89" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A90" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B90" s="7" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C90" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E90" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F90" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G90" s="18">
+        <v>130</v>
+      </c>
+      <c r="G90" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A91" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G91" s="18">
+        <v>130</v>
+      </c>
+      <c r="G91" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A92" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B92" s="7" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D92" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F92" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G92" s="18">
+        <v>130</v>
+      </c>
+      <c r="G92" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A93" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B93" s="7" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D93" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G93" s="18">
+        <v>130</v>
+      </c>
+      <c r="G93" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A94" s="7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B94" s="7" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D94" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E94" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F94" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G94" s="18">
+        <v>130</v>
+      </c>
+      <c r="G94" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A95" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B95" s="7" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G95" s="18">
+        <v>130</v>
+      </c>
+      <c r="G95" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A96" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E96" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F96" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G96" s="16">
+        <v>43788</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A97" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>463</v>
+      </c>
+      <c r="C97" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B96" s="7" t="s">
-        <v>464</v>
-      </c>
-      <c r="C96" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="D96" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E96" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="F96" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="G96" s="18">
+      <c r="D97" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E97" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G97" s="16">
         <v>43788</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A97" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="B97" s="7" t="s">
-        <v>465</v>
-      </c>
-      <c r="C97" s="7" t="s">
-        <v>446</v>
-      </c>
-      <c r="D97" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E97" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="F97" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G97" s="18">
-        <v>45761</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A98" s="7" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B98" s="7" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="C98" s="7" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D98" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E98" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F98" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F98" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G98" s="18">
+      <c r="G98" s="16">
         <v>45761</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A99" s="7" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B99" s="7" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C99" s="7" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E99" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F99" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F99" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G99" s="18">
+      <c r="G99" s="16">
         <v>45761</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A100" s="7" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B100" s="7" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="C100" s="7" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="D100" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E100" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F100" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F100" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G100" s="18">
+      <c r="G100" s="16">
         <v>45761</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A101" s="7" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B101" s="7" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C101" s="7" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E101" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F101" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F101" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G101" s="18">
+      <c r="G101" s="16">
         <v>45761</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A102" s="7" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B102" s="7" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C102" s="7" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E102" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F102" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="F102" s="8" t="s">
-        <v>341</v>
-      </c>
-      <c r="G102" s="18">
+      <c r="G102" s="16">
         <v>45761</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A103" s="7" t="s">
+        <v>444</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="C103" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E103" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="G103" s="16">
+        <v>45761</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A104" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C104" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E104" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="B103" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="C103" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E103" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F103" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G103" s="18">
+      <c r="F104" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G104" s="16">
         <v>44111</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A104" s="7"/>
-      <c r="B104" s="7"/>
-      <c r="C104" s="7"/>
-      <c r="D104" s="7"/>
-      <c r="E104" s="7"/>
-      <c r="F104" s="7" t="s">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A105" s="7"/>
+      <c r="B105" s="7"/>
+      <c r="C105" s="7"/>
+      <c r="D105" s="7"/>
+      <c r="E105" s="7"/>
+      <c r="F105" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G104" s="18">
-        <v>43788</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A105" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="B105" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="C105" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E105" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="F105" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G105" s="18">
+      <c r="G105" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A106" s="7" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B106" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D106" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F106" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G106" s="18">
+        <v>27</v>
+      </c>
+      <c r="G106" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A107" s="7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B107" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C107" s="7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D107" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F107" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G107" s="18">
+        <v>163</v>
+      </c>
+      <c r="G107" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A108" s="7" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D108" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G108" s="18">
+      <c r="G108" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A109" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="C109" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E109" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F109" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G109" s="16">
+        <v>43788</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A110" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="C110" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B109" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="C109" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="D109" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E109" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="F109" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G109" s="18">
+      <c r="D110" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E110" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F110" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="G110" s="16">
         <v>43788</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A110" s="7"/>
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
-      <c r="D110" s="7"/>
-      <c r="E110" s="7"/>
-      <c r="F110" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G110" s="18">
-        <v>43788</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A111" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="B111" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="C111" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="D111" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E111" s="7" t="s">
-        <v>173</v>
-      </c>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A111" s="7"/>
+      <c r="B111" s="7"/>
+      <c r="C111" s="7"/>
+      <c r="D111" s="7"/>
+      <c r="E111" s="7"/>
       <c r="F111" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G111" s="18">
+      <c r="G111" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A112" s="7" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D112" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E112" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G112" s="18">
+      <c r="G112" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A113" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B113" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F113" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G113" s="18">
+      <c r="G113" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A114" s="7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B114" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C114" s="7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D114" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E114" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F114" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G114" s="18">
+      <c r="G114" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A115" s="7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C115" s="7" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D115" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E115" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F115" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G115" s="18">
+      <c r="G115" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A116" s="7" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B116" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C116" s="7" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D116" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E116" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F116" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G116" s="18">
+      <c r="G116" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A117" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B117" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C117" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F117" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G117" s="18">
+      <c r="G117" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A118" s="7" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D118" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E118" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F118" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G118" s="18">
+      <c r="G118" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A119" s="7" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C119" s="7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D119" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E119" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G119" s="18">
+      <c r="G119" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A120" s="7" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D120" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E120" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F120" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G120" s="18">
+      <c r="G120" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A121" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B121" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C121" s="7" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D121" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F121" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G121" s="18">
+      <c r="G121" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A122" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D122" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F122" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G122" s="18">
+      <c r="G122" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A123" s="7" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D123" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E123" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F123" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G123" s="18">
+      <c r="G123" s="16">
         <v>43788</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="32" x14ac:dyDescent="0.8">
-      <c r="A124" s="9" t="s">
-        <v>359</v>
-      </c>
-      <c r="B124" s="11" t="s">
-        <v>360</v>
-      </c>
-      <c r="C124" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="D124" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E124" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="F124" s="11"/>
-      <c r="G124" s="20">
-        <v>45509</v>
+      <c r="A124" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B124" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D124" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E124" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="F124" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G124" s="16">
+        <v>43788</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A125" s="9" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C125" s="9" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="D125" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E125" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F125" s="11"/>
-      <c r="G125" s="20">
+      <c r="G125" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A126" s="9" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C126" s="9" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="D126" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E126" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F126" s="11"/>
-      <c r="G126" s="20">
+      <c r="G126" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A127" s="9" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C127" s="9" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F127" s="11"/>
-      <c r="G127" s="20">
+      <c r="G127" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A128" s="9" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="C128" s="9" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E128" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F128" s="11"/>
-      <c r="G128" s="20">
+      <c r="G128" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A129" s="9" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C129" s="9" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="D129" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E129" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F129" s="11"/>
-      <c r="G129" s="20">
+      <c r="G129" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A130" s="9" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C130" s="9" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="D130" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E130" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F130" s="11"/>
-      <c r="G130" s="20">
+      <c r="G130" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A131" s="9" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C131" s="9" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D131" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E131" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F131" s="11"/>
-      <c r="G131" s="20">
+      <c r="G131" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A132" s="9" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="C132" s="9" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="D132" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E132" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F132" s="11"/>
-      <c r="G132" s="20">
+      <c r="G132" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A133" s="9" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C133" s="9" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="D133" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E133" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F133" s="11"/>
-      <c r="G133" s="20">
+      <c r="G133" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A134" s="9" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C134" s="9" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F134" s="11"/>
-      <c r="G134" s="20">
+      <c r="G134" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A135" s="9" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C135" s="9" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="D135" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E135" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F135" s="11"/>
-      <c r="G135" s="20">
+      <c r="G135" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A136" s="9" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="C136" s="9" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="D136" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E136" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F136" s="11"/>
-      <c r="G136" s="20">
+      <c r="G136" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A137" s="9" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="B137" s="11" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="C137" s="9" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="D137" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E137" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F137" s="11"/>
-      <c r="G137" s="20">
+      <c r="G137" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A138" s="9" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="C138" s="9" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="D138" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E138" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F138" s="11"/>
-      <c r="G138" s="20">
+      <c r="G138" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A139" s="9" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="B139" s="11" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="C139" s="9" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="D139" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E139" s="9" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F139" s="11"/>
-      <c r="G139" s="20">
+      <c r="G139" s="17">
         <v>45509</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="32" x14ac:dyDescent="0.8">
       <c r="A140" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="B140" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="C140" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="D140" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E140" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="F140" s="11"/>
+      <c r="G140" s="17">
+        <v>45509</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A141" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="B141" s="11" t="s">
         <v>408</v>
       </c>
-      <c r="B140" s="11" t="s">
+      <c r="C141" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="C140" s="9" t="s">
-        <v>410</v>
-      </c>
-      <c r="D140" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E140" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="F140" s="11"/>
-      <c r="G140" s="20">
+      <c r="D141" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E141" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="F141" s="11"/>
+      <c r="G141" s="17">
         <v>45509</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A141" s="9" t="s">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A142" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="B142" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="C142" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="D142" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E142" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="F142" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G142" s="17">
+        <v>45715</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A143" s="9" t="s">
         <v>419</v>
       </c>
-      <c r="B141" s="11" t="s">
+      <c r="B143" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="C143" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="D143" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E143" s="9" t="s">
         <v>422</v>
       </c>
-      <c r="C141" s="9" t="s">
-        <v>421</v>
-      </c>
-      <c r="D141" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E141" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="F141" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="G141" s="20">
+      <c r="F143" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G143" s="17">
         <v>45715</v>
       </c>
     </row>
-    <row r="142" spans="1:7" ht="48" x14ac:dyDescent="0.8">
-      <c r="A142" s="9" t="s">
-        <v>420</v>
-      </c>
-      <c r="B142" s="9" t="s">
-        <v>427</v>
-      </c>
-      <c r="C142" s="9" t="s">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A144" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="B144" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="D142" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E142" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="F142" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="G142" s="20">
+      <c r="C144" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="D144" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E144" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="F144" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G144" s="17">
         <v>45715</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A143" s="9" t="s">
-        <v>418</v>
-      </c>
-      <c r="B143" s="11" t="s">
-        <v>425</v>
-      </c>
-      <c r="C143" s="9" t="s">
-        <v>426</v>
-      </c>
-      <c r="D143" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E143" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="F143" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="G143" s="20">
-        <v>45715</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.8">
-      <c r="A144" s="7"/>
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
-      <c r="D144" s="7"/>
-      <c r="E144" s="7"/>
-      <c r="F144" s="7"/>
-      <c r="G144" s="18"/>
-    </row>
-    <row r="145" spans="1:8" ht="32" x14ac:dyDescent="0.8">
-      <c r="A145" s="6" t="s">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A145" s="7"/>
+      <c r="B145" s="7"/>
+      <c r="C145" s="7"/>
+      <c r="D145" s="7"/>
+      <c r="E145" s="7"/>
+      <c r="F145" s="7"/>
+      <c r="G145" s="16"/>
+    </row>
+    <row r="146" spans="1:7" ht="32" x14ac:dyDescent="0.8">
+      <c r="A146" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B146" s="6"/>
+      <c r="C146" s="10"/>
+      <c r="D146" s="10"/>
+      <c r="E146" s="10"/>
+      <c r="F146" s="10"/>
+      <c r="G146" s="18"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A147" s="7" t="s">
         <v>199</v>
-      </c>
-      <c r="B145" s="6"/>
-      <c r="C145" s="10"/>
-      <c r="D145" s="10"/>
-      <c r="E145" s="10"/>
-      <c r="F145" s="10"/>
-      <c r="G145" s="21"/>
-    </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A146" s="7" t="s">
-        <v>200</v>
-      </c>
-      <c r="B146" s="7"/>
-      <c r="C146" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="D146" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E146" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F146" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G146" s="18">
-        <v>42507</v>
-      </c>
-    </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A147" s="7" t="s">
-        <v>58</v>
       </c>
       <c r="B147" s="7"/>
       <c r="C147" s="7" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D147" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E147" s="7" t="s">
-        <v>202</v>
+        <v>8</v>
       </c>
       <c r="F147" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="G147" s="18">
-        <v>41002</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.8">
+        <v>9</v>
+      </c>
+      <c r="G147" s="16">
+        <v>42507</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A148" s="7" t="s">
-        <v>205</v>
+        <v>58</v>
       </c>
       <c r="B148" s="7"/>
       <c r="C148" s="7" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D148" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E148" s="7" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="F148" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="G148" s="18">
+        <v>202</v>
+      </c>
+      <c r="G148" s="16">
         <v>41002</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.8">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A149" s="7" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B149" s="7"/>
       <c r="C149" s="7" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="D149" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E149" s="7" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="F149" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="G149" s="18">
+        <v>206</v>
+      </c>
+      <c r="G149" s="16">
         <v>41002</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.8">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A150" s="7" t="s">
-        <v>82</v>
+        <v>208</v>
       </c>
       <c r="B150" s="7"/>
       <c r="C150" s="7" t="s">
-        <v>320</v>
+        <v>211</v>
       </c>
       <c r="D150" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E150" s="7" t="s">
-        <v>83</v>
+        <v>209</v>
       </c>
       <c r="F150" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G150" s="18">
+        <v>210</v>
+      </c>
+      <c r="G150" s="16">
         <v>41002</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="48" x14ac:dyDescent="0.8">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A151" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B151" s="7" t="s">
-        <v>229</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B151" s="7"/>
       <c r="C151" s="7" t="s">
-        <v>97</v>
+        <v>319</v>
       </c>
       <c r="D151" s="7" t="s">
         <v>13</v>
       </c>
       <c r="E151" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F151" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="G151" s="16">
+        <v>41002</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" ht="48" x14ac:dyDescent="0.8">
+      <c r="A152" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B152" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C152" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D152" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E152" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F151" s="7" t="s">
+      <c r="F152" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G151" s="18">
+      <c r="G152" s="16">
         <v>42118</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A152"/>
-      <c r="B152"/>
-      <c r="C152"/>
-      <c r="D152"/>
-      <c r="E152"/>
-      <c r="F152"/>
-      <c r="G152" s="22"/>
-    </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A153" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B153" s="2"/>
-      <c r="C153" s="3"/>
-      <c r="D153" s="3"/>
-      <c r="E153" s="3"/>
-      <c r="F153" s="3"/>
-      <c r="G153" s="23"/>
-    </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.8">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A153"/>
+      <c r="B153"/>
+      <c r="C153"/>
+      <c r="D153"/>
+      <c r="E153"/>
+      <c r="F153"/>
+      <c r="G153" s="19"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A154" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B154" s="2"/>
       <c r="C154" s="3"/>
       <c r="D154" s="3"/>
       <c r="E154" s="3"/>
       <c r="F154" s="3"/>
-      <c r="G154" s="23"/>
-    </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A155" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="B155" s="3"/>
+      <c r="G154" s="20"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A155" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B155" s="2"/>
       <c r="C155" s="3"/>
       <c r="D155" s="3"/>
       <c r="E155" s="3"/>
       <c r="F155" s="3"/>
-      <c r="G155" s="23"/>
-    </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.8">
+      <c r="G155" s="20"/>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.8">
       <c r="A156" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
       <c r="D156" s="3"/>
       <c r="E156" s="3"/>
       <c r="F156" s="3"/>
-      <c r="G156" s="23"/>
-    </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="A157" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="B157" s="5"/>
-      <c r="C157" s="5"/>
-      <c r="D157" s="5"/>
-      <c r="E157" s="5"/>
-      <c r="F157" s="5"/>
-    </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.8">
-      <c r="H160" s="4"/>
+      <c r="G156" s="20"/>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A157" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B157" s="3"/>
+      <c r="C157" s="3"/>
+      <c r="D157" s="3"/>
+      <c r="E157" s="3"/>
+      <c r="F157" s="3"/>
+      <c r="G157" s="20"/>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.8">
+      <c r="A158" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="5"/>
+      <c r="F158" s="5"/>
+    </row>
+    <row r="161" spans="8:8" x14ac:dyDescent="0.8">
+      <c r="H161" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F77" r:id="rId1" display="murakami.shinya@jaxa.jp" xr:uid="{01DA75B4-19A0-4336-8C87-BE018A8D132A}"/>
-    <hyperlink ref="F62" r:id="rId2" display="murakami.shinya@jaxa.jp" xr:uid="{D1657E2D-7AB0-4C53-B977-119F78918607}"/>
-    <hyperlink ref="F47" r:id="rId3" display="murakami.shinya@jaxa.jp" xr:uid="{C81BC639-28AF-4159-B44A-854ED34AE89C}"/>
-    <hyperlink ref="F75" r:id="rId4" display="murakami.shinya@jaxa.jp" xr:uid="{7F077A21-6A46-4357-819D-567BD3D440C0}"/>
-    <hyperlink ref="F76" r:id="rId5" display="murakami.shinya@jaxa.jp" xr:uid="{E25FB432-2C67-446C-877E-ED14B3BB1D3C}"/>
-    <hyperlink ref="F97" r:id="rId6" display="murakami.shinya@jaxa.jp" xr:uid="{F3720F63-95ED-4C8F-9B54-81C948F40B00}"/>
-    <hyperlink ref="F99" r:id="rId7" display="murakami.shinya@jaxa.jp" xr:uid="{5138A935-04AD-468A-B5D1-85FCA7D8FB22}"/>
-    <hyperlink ref="F98" r:id="rId8" display="murakami.shinya@jaxa.jp" xr:uid="{5725B4D5-AC59-40E6-9B3A-ADCB5EB0C6D8}"/>
-    <hyperlink ref="F102" r:id="rId9" display="murakami.shinya@jaxa.jp" xr:uid="{1CB633E2-E1AB-437B-B517-B9F5687F978C}"/>
-    <hyperlink ref="F100" r:id="rId10" display="murakami.shinya@jaxa.jp" xr:uid="{EF3A89FD-08B4-46C1-BD91-0D95801E70FD}"/>
-    <hyperlink ref="F101" r:id="rId11" display="murakami.shinya@jaxa.jp" xr:uid="{12C0759C-69E8-43C4-9941-4C2A0856C253}"/>
-    <hyperlink ref="F46" r:id="rId12" display="murakami.shinya@jaxa.jp" xr:uid="{7A172708-FC01-4F69-BED7-7CAC90640566}"/>
+    <hyperlink ref="F78" r:id="rId1" display="murakami.shinya@jaxa.jp" xr:uid="{01DA75B4-19A0-4336-8C87-BE018A8D132A}"/>
+    <hyperlink ref="F63" r:id="rId2" display="murakami.shinya@jaxa.jp" xr:uid="{D1657E2D-7AB0-4C53-B977-119F78918607}"/>
+    <hyperlink ref="F48" r:id="rId3" display="murakami.shinya@jaxa.jp" xr:uid="{C81BC639-28AF-4159-B44A-854ED34AE89C}"/>
+    <hyperlink ref="F76" r:id="rId4" display="murakami.shinya@jaxa.jp" xr:uid="{7F077A21-6A46-4357-819D-567BD3D440C0}"/>
+    <hyperlink ref="F77" r:id="rId5" display="murakami.shinya@jaxa.jp" xr:uid="{E25FB432-2C67-446C-877E-ED14B3BB1D3C}"/>
+    <hyperlink ref="F98" r:id="rId6" display="murakami.shinya@jaxa.jp" xr:uid="{F3720F63-95ED-4C8F-9B54-81C948F40B00}"/>
+    <hyperlink ref="F100" r:id="rId7" display="murakami.shinya@jaxa.jp" xr:uid="{5138A935-04AD-468A-B5D1-85FCA7D8FB22}"/>
+    <hyperlink ref="F99" r:id="rId8" display="murakami.shinya@jaxa.jp" xr:uid="{5725B4D5-AC59-40E6-9B3A-ADCB5EB0C6D8}"/>
+    <hyperlink ref="F103" r:id="rId9" display="murakami.shinya@jaxa.jp" xr:uid="{1CB633E2-E1AB-437B-B517-B9F5687F978C}"/>
+    <hyperlink ref="F101" r:id="rId10" display="murakami.shinya@jaxa.jp" xr:uid="{EF3A89FD-08B4-46C1-BD91-0D95801E70FD}"/>
+    <hyperlink ref="F102" r:id="rId11" display="murakami.shinya@jaxa.jp" xr:uid="{12C0759C-69E8-43C4-9941-4C2A0856C253}"/>
+    <hyperlink ref="F47" r:id="rId12" display="murakami.shinya@jaxa.jp" xr:uid="{7A172708-FC01-4F69-BED7-7CAC90640566}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="54" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId13"/>

</xml_diff>